<commit_message>
Se agregó la funcionalidad para ajustar el ancho de las columnas en el excel
</commit_message>
<xml_diff>
--- a/data/clean/Celulares_20260609.xlsx
+++ b/data/clean/Celulares_20260609.xlsx
@@ -1692,6 +1692,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F144"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="75.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="75.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">

</xml_diff>